<commit_message>
docs(qa): Author 54-case suite and adopt no-fabrication hardening
Phase 6: real 54-case workbook replacing placeholders, with exact
module (8/4/10/6/12/5/4/3/2) and type (20/14/6/5/4/2/3) distribution,
TC-COMP-001 for cross-browser parity, past-date framed as a recorded
probe, and all 20 DRS requirements covered. All cases Not Run.

Also adopt concurrent hardening: 20-REQ DRS, estimate-free status
language, corrected boundary data, Firefox as primary browser, and
installer-gated scope freeze with no silent redistribution.
</commit_message>
<xml_diff>
--- a/docs/04-test-cases/test-cases.xlsx
+++ b/docs/04-test-cases/test-cases.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,7 +479,22 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>Status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Defect ID</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -496,17 +511,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Scenario 1</t>
+          <t>Valid login</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify admin logs in with valid credentials and lands on Dashboard</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -521,34 +536,37 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Instance installed; qa_admin provisioned</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>users.md qa_admin</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open SUT URL 2. Enter qa_admin username 3. Enter password 4. Click Login</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Dashboard loads &lt;5s; user menu shows admin; session established</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -558,22 +576,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>REQ-AUTH-001</t>
+          <t>REQ-AUTH-002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Scenario 2</t>
+          <t>Valid login</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify ESS user logs in and sees role-assigned modules only</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -588,34 +606,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess linked to employee record</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>users.md qa_ess</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open SUT URL 2. Enter qa_ess username 3. Enter password 4. Click Login 5. Inspect side menu</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>ESS landing shown; PIM/Leave visible; Admin menu absent</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -625,22 +646,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>REQ-AUTH-001</t>
+          <t>REQ-AUTH-003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Scenario 3</t>
+          <t>Invalid login</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify wrong password is rejected with a message and no session</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -650,39 +671,42 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_admin exists</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>qa_admin + wrong password</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open SUT URL 2. Enter qa_admin username 3. Enter wrong password 4. Click Login 5. Try dashboard URL directly</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Stays on login + error message; direct dashboard URL redirects to login</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -692,22 +716,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>REQ-AUTH-001</t>
+          <t>REQ-AUTH-003</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Scenario 4</t>
+          <t>Invalid login</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify unknown username is rejected without revealing account existence</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -717,39 +741,42 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Fresh session</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>ghost_user_999 (synthetic)</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open SUT URL 2. Enter unknown username 3. Enter any password 4. Click Login</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Login rejected with generic message; no session created</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -759,64 +786,67 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>REQ-AUTH-001</t>
+          <t>REQ-AUTH-003</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Scenario 5</t>
+          <t>Empty login</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify empty username / password / both are rejected inline</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Fresh session</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>empty-string attempts x3</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Submit with empty username 2. Submit with empty password 3. Submit both empty</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Inline required messages each time; no session; no server error page</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -826,64 +856,67 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>REQ-AUTH-001</t>
+          <t>REQ-AUTH-003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Scenario 6</t>
+          <t>Whitespace login</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify whitespace-only credentials are treated as empty/invalid</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Fresh session</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>three-space strings</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Enter spaces in both fields 2. Click Login</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Rejected as empty/invalid with message; no session</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -893,22 +926,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>REQ-AUTH-001</t>
+          <t>REQ-AUTH-004</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Scenario 7</t>
+          <t>Logout</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify logout terminates session and returns to login</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -923,34 +956,37 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged in as qa_admin</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>active session</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Click user menu 2. Click Logout 3. Observe landing page</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Login page shown; session cookie invalidated</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -960,22 +996,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>REQ-AUTH-001</t>
+          <t>REQ-AUTH-004</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Authentication</t>
+          <t>Auth</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Scenario 8</t>
+          <t>Session</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify back-button and direct URL after logout cannot re-enter</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -985,39 +1021,42 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>State</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Just logged out (TC-AUTH-007)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>expired session</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Press browser Back 2. Paste dashboard URL directly 3. Attempt an action</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Redirect to login; no authenticated content or action possible</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1037,17 +1076,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Scenario 9</t>
+          <t>Load</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify dashboard widgets load completely without errors</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1057,34 +1096,37 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged in as qa_admin</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>default dashboard</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Log in 2. Wait for dashboard 3. Scroll all widgets</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>All widgets render &lt;5s; no stuck spinners; record console errors if any</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1104,22 +1146,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Scenario 10</t>
+          <t>Navigation</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify primary nav links route to the correct modules</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1129,29 +1171,32 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>nav map</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Click each primary nav item 2. Check module header per landing</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Each link lands on its matching module; labels consistent</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1171,54 +1216,57 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Scenario 11</t>
+          <t>Cross-browser</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify dashboard identical in Chrome vs Firefox at 1920x1080</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Compatibility</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged in on both browsers</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>same account</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open dashboard in Chrome 2. Open in Firefox 3. Compare widgets/order/layout</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M12" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Same widgets and order; no layout break or missing control</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1228,7 +1276,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>REQ-DASH-001</t>
+          <t>REQ-AUTH-004</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1238,12 +1286,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Scenario 12</t>
+          <t>Session</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify unauthenticated dashboard URL redirects to login</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1253,39 +1301,42 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged out</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>dashboard URL</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Ensure logged out 2. Paste dashboard URL 3. Submit</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Redirect to login page; no dashboard content exposed</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1305,12 +1356,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Scenario 13</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify employee created with valid data appears in list with ID</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1325,34 +1376,37 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged in as admin</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>valid_employee.csv E2001</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. PIM &gt; Add Employee 2. Fill first/last/ID/DOB 3. Save 4. Search ID in list</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Record appears with ID E2001; detail matches input</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1362,7 +1416,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>REQ-PIM-001</t>
+          <t>REQ-PIM-004</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1372,12 +1426,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Scenario 14</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify missing required fields and duplicate IDs are blocked, never silently saved</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1387,39 +1441,42 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged in as admin</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>invalid_employee.csv empty row + duplicate E2001</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. PIM &gt; Add 2. Leave required empty 3. Save 4. Retry with existing ID E2001 5. Search to confirm no second record</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Inline errors for both attempts; no record created; no duplicate E2001 (search confirms)</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1439,54 +1496,57 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Scenario 15</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify 50-char first name accepted at max boundary</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged in as admin</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>boundary_employee.csv E2005</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. PIM &gt; Add 2. Enter 50-char name 3. Save 4. Note 51-char behavior if testable</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>50-char saved; over-limit outcome recorded as observed</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1496,7 +1556,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>REQ-PIM-001</t>
+          <t>REQ-PIM-002</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1506,12 +1566,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Scenario 16</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify exact first-name search returns exactly one hit</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1526,34 +1586,37 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>E2001 exists</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>search_test_data.csv Aarav</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. PIM &gt; Employee List 2. Search 'Aarav' 3. Reset</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Exactly the E2001 row; Reset restores full list</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1563,7 +1626,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>REQ-PIM-001</t>
+          <t>REQ-PIM-002</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1573,22 +1636,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Scenario 17</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify no-match search shows empty state, not stale rows</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1598,29 +1661,32 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>search_test_data.csv ZzzNoMatch</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Search 'ZzzNoMatch' 2. Observe list 3. Clear search</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Empty-list message; no stale rows; clear restores list</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1630,7 +1696,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>REQ-PIM-001</t>
+          <t>REQ-PIM-002</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1640,54 +1706,57 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Scenario 18</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify case/partial/whitespace search behaves sanely</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>E2001 exists</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>search_test_data.csv aarav/Aar/trail-space</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Search 'aarav' 2. Search 'Aar' 3. Search 'Sharma ' 4. Record each rule</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Behavior matches observed rule; any deviation is a finding</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1697,7 +1766,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>REQ-PIM-001</t>
+          <t>REQ-PIM-003</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1707,17 +1776,17 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Scenario 19</t>
+          <t>View</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify employee detail view shows stored data</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1727,34 +1796,37 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>E2001 exists</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>E2001</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open E2001 from list 2. Compare fields to creation input</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>All fields match creation data</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1764,7 +1836,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>REQ-PIM-001</t>
+          <t>REQ-PIM-003</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1774,17 +1846,17 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Scenario 20</t>
+          <t>Delete</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify employee delete with confirmation removes the record</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1794,34 +1866,37 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>E2009 exists (disposable); delete available</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>invalid_employee.csv E2009</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Select record 2. Delete 3. Confirm 4. Search ID</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Confirm dialog shown; record gone; search finds nothing</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1831,7 +1906,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>REQ-PIM-001</t>
+          <t>REQ-PIM-002</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1841,54 +1916,57 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Scenario 21</t>
+          <t>Pagination</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify list pagination keeps filter context and counts</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>&gt;=2 pages of employees</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>seeded list</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Apply filter 2. Go to page 2 3. Check counts</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Filter retained; counts consistent across pages</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1898,7 +1976,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>REQ-PIM-001</t>
+          <t>REQ-PIM-002</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1908,22 +1986,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Scenario 22</t>
+          <t>Table</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify list table columns and row actions are consistent</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1933,29 +2011,32 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>employee list</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Inspect headers 2. Check row actions 3. Resize to 1920</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Uniform headers/actions; no truncation hiding actions</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1975,12 +2056,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Scenario 23</t>
+          <t>Edit</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify edited personal info saves and persists after refresh</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1995,34 +2076,37 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>E2001 exists</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>edited contact fields</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open E2001 profile 2. Edit contact info 3. Save 4. Refresh 5. Reopen</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Saved confirmation; values persist post-refresh</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2042,54 +2126,57 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Scenario 24</t>
+          <t>Validation</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify invalid date format is rejected and not saved</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>E2001 exists</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>not-a-date</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open profile 2. Enter 'not-a-date' in date field 3. Save 4. Refresh</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Field error; original value retained after refresh</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2109,54 +2196,57 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Scenario 25</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify age boundaries: 18y accepted, future DOB rejected</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged in as admin</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>boundary E2006/E2007 + future E2010</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Set DOB 2008-10-03 2. Set DOB 1926-10-03 3. Set DOB 2030-01-01</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Boundary DOBs accepted per policy; future DOB rejected with message</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2176,54 +2266,57 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Scenario 26</t>
+          <t>Form UI</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify required markers, dropdowns and error placement are consistent</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Profile open</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>profile form</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Scan required markers 2. Open each dropdown 3. Trigger one error</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>All required marked; errors adjacent to fields; dropdowns operable</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2243,17 +2336,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Scenario 27</t>
+          <t>Reset</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify Reset discards unsaved edits and restores originals</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2263,34 +2356,37 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>E2001 exists</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>dirty form</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Edit two fields 2. Click Reset 3. Read values</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Original values restored; nothing saved</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2310,22 +2406,22 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Scenario 28</t>
+          <t>Keyboard</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify profile form fully operable by keyboard with visible focus</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2335,29 +2431,32 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>keyboard only</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Tab through entire form 2. Fill and save without mouse</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Logical tab order; focus always visible; save succeeds</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2377,12 +2476,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Scenario 29</t>
+          <t>Apply</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify full-day leave with valid type/date/balance submits as Pending</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2397,34 +2496,37 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess with Annual balance</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>leave-data.csv valid row</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Login ESS 2. Leave &gt; Apply 3. Pick Annual 4. Check balance 5. Future working day 6. Full Day 7. Comment 8. Apply</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Accepted; appears in My Leave with initial Pending status</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2434,7 +2536,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-002</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2444,12 +2546,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Scenario 30</t>
+          <t>Apply</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify morning half-day submits with half duration</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2464,34 +2566,37 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess with balance</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>2030-06-02 Half Day - Morning</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Apply 2. Half Day 3. Morning 4. Submit 5. Check record</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Recorded as 0.5 day against balance</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2501,7 +2606,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-002</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2511,17 +2616,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Scenario 31</t>
+          <t>Apply</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify specific-time leave submits with start/end times</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2531,34 +2636,37 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess with balance</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>09:00-13:00 window</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Apply 2. Specify Time 3. Enter range 4. Submit</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Start/end stored and shown on the record</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2568,7 +2676,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-002</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2578,54 +2686,57 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Scenario 32</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify today-date and far-future single day are accepted</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess with balance</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>2026-10-03 + 2030-06-02</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Apply for today 2. Apply for 2030-06-02 3. Record weekend-policy hits</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Both accepted unless a stated policy blocks; policy recorded</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2635,7 +2746,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-003</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2645,12 +2756,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Scenario 33</t>
+          <t>Invalid</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify End-before-Start range is rejected before submit</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2660,39 +2771,42 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess logged in</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>leave_boundary_dates.csv end-before-start</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Apply 2. From 2030-06-05 To 2030-06-04 3. Submit</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Rejected with date-order message; nothing in history</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2702,7 +2816,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-003</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2712,12 +2826,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Scenario 34</t>
+          <t>Probe</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Probe past-date submission and record the observed policy without assuming it</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -2727,39 +2841,42 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess logged in</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>leave_boundary_dates.csv past-date-probe</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Apply 2. Enter past date 2020-01-15 3. Submit 4. Record outcome vs any stated policy</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Either blocked with a message or accepted into history; outcome recorded as observed policy — no defect asserted without an authoritative rule</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2769,7 +2886,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-005</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2779,12 +2896,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Scenario 35</t>
+          <t>Balance</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify insufficient/zero balance is rejected or flagged per config</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -2794,39 +2911,42 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess with exhausted type</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>zero-balance type</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Apply 2. Pick exhausted type 3. Check balance 4. Submit</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M36" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Rejected or warned per configuration; actual behavior recorded</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2836,7 +2956,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-005</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2846,54 +2966,57 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Scenario 36</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify missing leave type is rejected as required</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess logged in</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>empty type</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Apply 2. Skip type 3. Fill dates 4. Submit</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Required-field message; no submission</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2903,7 +3026,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-004</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2913,12 +3036,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Scenario 37</t>
+          <t>Cancel</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify pending request can be cancelled with status update</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2928,39 +3051,42 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>State</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Pending request exists</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>TC-LEAVE-001 record</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. My Leave 2. Select pending 3. Cancel 4. Confirm</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M38" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Status Cancelled; balance handling recorded as observed</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2970,7 +3096,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-004</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2980,12 +3106,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Scenario 38</t>
+          <t>Approve</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify admin approval moves Pending to Approved</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2995,39 +3121,42 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>State</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Pending request; admin session</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>pending record</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Login admin 2. Leave List 3. Approve 4. Check employee view</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Status Approved in both views</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3037,7 +3166,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-004</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -3047,17 +3176,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Scenario 39</t>
+          <t>Reject</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify admin rejection moves Pending to Rejected with comment</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3067,34 +3196,37 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Pending request; admin session</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>pending record + comment</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Login admin 2. Leave List 3. Reject with comment</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Status Rejected; comment visible to employee</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3104,7 +3236,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>REQ-LEAVE-001</t>
+          <t>REQ-LEAVE-004</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -3114,54 +3246,57 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Scenario 40</t>
+          <t>Invalid transition</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify approved-to-modify and rejected-to-cancel are blocked</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>State</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Approved + Rejected records exist</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>decided records</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Try modify approved 2. Try cancel rejected 3. Record outcomes</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Actions unavailable or rejected with message</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3181,17 +3316,17 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Scenario 41</t>
+          <t>Clock in</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify clock-in creates an attendance record with timestamp</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3201,34 +3336,37 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>qa_ess; Time present</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>punch time</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Time &gt; Attendance 2. Clock In 3. Check record</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Record with correct timestamp appears</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3248,17 +3386,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Scenario 42</t>
+          <t>Clock out</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify clock-out completes the record with computed duration</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3268,34 +3406,37 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Clocked-in session</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>same shift</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Clock Out 2. Open record 3. Read duration</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M43" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>End time + duration recorded and correct</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3315,54 +3456,57 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Scenario 43</t>
+          <t>Sequence</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify clock-out without clock-in is rejected</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>No open punch</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>idle attendance</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Attempt Clock Out with no open punch</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M44" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Message shown; no orphan record created</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3382,22 +3526,22 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Scenario 44</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify duplicate/out-of-order punches are handled per observed rule</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -3407,29 +3551,32 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>double punch</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Clock In twice 2. Backdate a punch 3. Record rule</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Rejected or merged per observed rule; recorded</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3449,17 +3596,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Scenario 45</t>
+          <t>Timesheet</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify timesheet filter narrows and data persists after refresh</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3469,34 +3616,37 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Records exist</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>date filter</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open timesheet 2. Filter by date 3. Refresh 4. Re-check</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Filter narrows correctly; data survives refresh</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3516,17 +3666,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Scenario 46</t>
+          <t>Create</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify vacancy with required fields appears in list</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3536,34 +3686,37 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Admin; Recruitment present</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>QA Engineer vacancy</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Recruitment &gt; Vacancies 2. Add 3. Fill required 4. Save</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Vacancy listed with entered details</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3583,54 +3736,57 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Scenario 47</t>
+          <t>Required</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify vacancy missing required fields is blocked</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>empty title</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Add vacancy 2. Skip title 3. Save</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Inline errors; nothing created</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3650,54 +3806,57 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Scenario 48</t>
+          <t>Hiring step</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify candidate status advances with history kept</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>State</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Vacancy + candidate exist</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>candidate record</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Open candidate 2. Advance one hiring step 3. Check history</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M49" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Status updated; prior step retained in history</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3717,54 +3876,57 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Scenario 49</t>
+          <t>Cross-browser</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify vacancy search matches on second browser</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Compatibility</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Vacancy exists</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>search term</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Search in Chrome 2. Repeat in Firefox 3. Compare</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M50" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Identical result sets and order</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3774,7 +3936,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>REQ-REP-001</t>
+          <t>REQ-REPORT-001</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -3784,17 +3946,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Scenario 50</t>
+          <t>Generate</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify filtered report returns matching rows</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3804,34 +3966,37 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Employees + leave exist</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>PIM filter set</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Reports 2. Pick report 3. Set filters 4. Run</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Rows match filters; counts sane</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3841,7 +4006,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>REQ-REP-001</t>
+          <t>REQ-REPORT-001</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -3851,22 +4016,22 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Scenario 51</t>
+          <t>Empty</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify impossible filter combo shows empty state, not an error</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3876,29 +4041,32 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>impossible combo</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Set mutually-exclusive filters 2. Run</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M52" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Empty-state message; no error page or stale data</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3908,7 +4076,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>REQ-REP-001</t>
+          <t>REQ-REPORT-001</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -3918,17 +4086,17 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Scenario 52</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify report export downloads a file matching on-screen rows</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3938,34 +4106,37 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Report with rows; export present</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>generated report</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Run report 2. Export 3. Open file 4. Compare counts</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M53" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>File downloads; row count matches screen</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3980,126 +4151,132 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>UI/Compat</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Scenario 53</t>
+          <t>Keyboard path</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify keyboard-only login to dashboard to logout works end to end</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Accessibility</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Fresh session</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>keyboard only</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Tab to username/password/Login 2. Navigate dashboard 3. Logout via keyboard</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>Full path completable; focus visible throughout</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TC-UI-002</t>
+          <t>TC-COMP-001</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>REQ-UI-001</t>
+          <t>REQ-COMP-001</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>UI/Compat</t>
+          <t>Compatibility</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Scenario 54</t>
+          <t>Brand parity</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Title per design standard</t>
+          <t>Verify header/footer/branding identical across modules and browsers</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Compatibility</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Logged in</t>
+          <t>Logged in both browsers</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>Synthetic</t>
+          <t>4+ modules</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Firefox/Chromium 1920x1080</t>
+          <t>OrangeHRM 5.8.1 self-hosted; Firefox155 primary / Chrome153 secondary; 1920x1080</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>1.Login 2.Navigate 3.Act 4.Verify</t>
+          <t>1. Visit 4 modules in Firefox 2. Repeat in Chrome 3. Compare chrome</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Expected per DRS</t>
-        </is>
-      </c>
-      <c r="M55" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
+          <t>No branding/layout drift between modules or browsers</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr"/>
+      <c r="P55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(qa): Resolve planned-input dispute by conforming E2001 rerun
Seed E2001 (Aarav Sharma, DOB 1990-01-15) and rerun TC-PIM-001/002/004/005/007
with specified data: all five pass with evidence. Restores 17/2/2/33 across
execution log, case workbook, RTM, summary, and final report (all verified in
sync; Expected column frozen since authoring). Corrects the record: free-text
name queries are submitted as filters (ZzzNoMatch -> empty state). Zero SUT
defects stands.
</commit_message>
<xml_diff>
--- a/docs/04-test-cases/test-cases.xlsx
+++ b/docs/04-test-cases/test-cases.xlsx
@@ -559,14 +559,21 @@
           <t>Dashboard loads &lt;5s; user menu shows admin; session established</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Login page HTTP 200/title OrangeHRM with username+password+Login; qa_admin login lands /dashboard/index &lt;5s with admin user menu</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-AUTH-001-login-page.png + TC-AUTH-002-admin-dashboard.png</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -629,14 +636,21 @@
           <t>ESS landing shown; PIM/Leave visible; Admin menu absent</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>ESS login lands /dashboard/index with restricted 8-item nav (Leave/Time/My Info/Performance/Dashboard/Directory/Claim/Buzz); Admin+PIM+Recruitment+Maintenance absent. Expected text says "PIM/Leave visible" — PIM is correctly hidden for ESS; test-design wording needs correction, NOT an SUT defect. No BUG filed.</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-AUTH-002-ess-dashboard.png; TEST-DESIGN issue flagged, Expected frozen per process</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -699,14 +713,21 @@
           <t>Stays on login + error message; direct dashboard URL redirects to login</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Wrong password rejected; stays on /auth/login with "Invalid credentials" toast; no session</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-AUTH-003-invalid-password.png</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -769,14 +790,21 @@
           <t>Login rejected with generic message; no session created</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Unknown username rejected with generic "Invalid credentials" (same as wrong password — no account enumeration); stays on login, no session</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-AUTH-004-unknown-user.png</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -839,14 +867,21 @@
           <t>Inline required messages each time; no session; no server error page</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Empty username+password rejected inline with "Required" x2; stays on login, no session</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-AUTH-005-empty-credentials.png</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -909,14 +944,21 @@
           <t>Rejected as empty/invalid with message; no session</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Whitespace-only credentials treated as empty: "Required" x2 shown; stays on login, no session</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-AUTH-006-whitespace-credentials.png</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -979,14 +1021,21 @@
           <t>Login page shown; session cookie invalidated</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Logout via user menu returns to /auth/login</t>
+        </is>
+      </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-AUTH-007-after-logout.png</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1049,14 +1098,21 @@
           <t>Redirect to login; no authenticated content or action possible</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Browser Back + direct /dashboard/index after logout both land on /auth/login; no authenticated content or action possible</t>
+        </is>
+      </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-AUTH-008-back-button.png + TC-DASH-004-direct-url-after-logout.png</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1119,14 +1175,21 @@
           <t>All widgets render &lt;5s; no stuck spinners; record console errors if any</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Admin dashboard loads with 12-item nav (Admin/PIM/Leave/Time/Recruitment/My Info/Performance/Dashboard/Directory/Maintenance/Claim/Buzz); ESS dashboard loads with 8-item restricted nav</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-DASH-001-dashboard-load.png + TC-AUTH-002-*-dashboard.png</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1189,14 +1252,21 @@
           <t>Each link lands on its matching module; labels consistent</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>PIM/Leave/Time/Recruitment nav targets each land on matching module (h6 PIM/Leave/Time+Timesheets/Recruitment)</t>
+        </is>
+      </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-DASH-002-nav-recruitment.png</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1259,14 +1329,11 @@
           <t>Same widgets and order; no layout break or missing control</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1329,14 +1396,21 @@
           <t>Redirect to login page; no dashboard content exposed</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Unauthenticated /dashboard/index redirects to /auth/login; no dashboard content exposed</t>
+        </is>
+      </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-DASH-004-direct-url-after-logout.png</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1399,14 +1473,21 @@
           <t>Record appears with ID E2001; detail matches input</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr"/>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>E2001 (Aarav Sharma, DOB 1990-01-15 per valid_employee.csv) saved ("Successfully Saved"), found by ID search (1 card), DOB persists after refresh. Conforming rerun 2026-10-03; exploratory E2091 probe retained as supporting evidence.</t>
+        </is>
+      </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-PIM-001-E2001-saved.png + TC-PIM-001-E2001-in-list.png + TC-PIM-007-E2001-detail.png</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1469,14 +1550,21 @@
           <t>Inline errors for both attempts; no record created; no duplicate E2001 (search confirms)</t>
         </is>
       </c>
-      <c r="M15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Empty-required blocked inline ("Required" x2, stays on form); duplicate E2001 blocked ("Employee Id already exists"); ID search confirms still exactly 1 E2001 record — no silent save, no duplicate. Conforming rerun 2026-10-03.</t>
+        </is>
+      </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-PIM-002-E2001-duplicate.png</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1539,14 +1627,21 @@
           <t>50-char saved; over-limit outcome recorded as observed</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr"/>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Assumed 50-char max is wrong: 50-char rejected, and true limit observed at 30 ("Should not exceed 30 characters"); 30-char accepted+saved+retrievable (E2092), 31-char rejected. App validation correct and consistent — test-design assumption needs correction, NOT an SUT defect. No BUG filed.</t>
+        </is>
+      </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
+          <t>Fail</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-PIM-003-true-boundary-30-31.png; Expected frozen per process</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1609,14 +1704,21 @@
           <t>Exactly the E2001 row; Reset restores full list</t>
         </is>
       </c>
-      <c r="M17" t="inlineStr"/>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Name autocomplete suggests Aarav; select+Search returns exactly 1 card (E2001 Aarav Sharma); Reset restores full list (6 cards). Conforming rerun 2026-10-03 with search_test_data.csv 'Aarav'.</t>
+        </is>
+      </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-PIM-004-Aarav-search.png</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1679,14 +1781,21 @@
           <t>Empty-list message; no stale rows; clear restores list</t>
         </is>
       </c>
-      <c r="M18" t="inlineStr"/>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Name query 'ZzzNoMatch' returns 0 cards with 'No Records Found' empty state — no stale rows. Conforming rerun 2026-10-03; free text IS submitted as a filter (earlier select-only theory disproven).</t>
+        </is>
+      </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-PIM-005-ZzzNoMatch.png</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1749,14 +1858,11 @@
           <t>Behavior matches observed rule; any deviation is a finding</t>
         </is>
       </c>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1819,14 +1925,21 @@
           <t>All fields match creation data</t>
         </is>
       </c>
-      <c r="M20" t="inlineStr"/>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>E2001 detail shows stored creation data (Aarav Sharma, E2001, DOB 1990-01-15 persists after save+refresh). Conforming rerun 2026-10-03.</t>
+        </is>
+      </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr"/>
-      <c r="P20" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-PIM-007-E2001-detail.png</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1889,14 +2002,11 @@
           <t>Confirm dialog shown; record gone; search finds nothing</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1959,14 +2069,11 @@
           <t>Filter retained; counts consistent across pages</t>
         </is>
       </c>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2029,14 +2136,11 @@
           <t>Uniform headers/actions; no truncation hiding actions</t>
         </is>
       </c>
-      <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2099,14 +2203,11 @@
           <t>Saved confirmation; values persist post-refresh</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2169,14 +2270,11 @@
           <t>Field error; original value retained after refresh</t>
         </is>
       </c>
-      <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2239,14 +2337,11 @@
           <t>Boundary DOBs accepted per policy; future DOB rejected with message</t>
         </is>
       </c>
-      <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2309,14 +2404,11 @@
           <t>All required marked; errors adjacent to fields; dropdowns operable</t>
         </is>
       </c>
-      <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2379,14 +2471,11 @@
           <t>Original values restored; nothing saved</t>
         </is>
       </c>
-      <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2449,14 +2538,11 @@
           <t>Logical tab order; focus always visible; save succeeds</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr"/>
-      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2519,14 +2605,21 @@
           <t>Accepted; appears in My Leave with initial Pending status</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr"/>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>ESS Apply Leave renders "No Leave Types with Leave Balance" — submission preconditions (leave type + entitlement/balance for qa_ess) not configured in this cycle; cannot assert submit behaviour</t>
+        </is>
+      </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O30" t="inlineStr"/>
-      <c r="P30" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-LEAVE-002-ess-apply-form.png; precondition: provision leave entitlement then re-execute</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2589,14 +2682,21 @@
           <t>Recorded as 0.5 day against balance</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr"/>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Same entitlement precondition as TC-LEAVE-001; half-day submit not attemptable</t>
+        </is>
+      </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>evidence/smoke/TC-LEAVE-002-ess-apply-form.png</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2659,14 +2759,11 @@
           <t>Start/end stored and shown on the record</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2729,14 +2826,11 @@
           <t>Both accepted unless a stated policy blocks; policy recorded</t>
         </is>
       </c>
-      <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2799,14 +2893,11 @@
           <t>Rejected with date-order message; nothing in history</t>
         </is>
       </c>
-      <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2869,14 +2960,11 @@
           <t>Either blocked with a message or accepted into history; outcome recorded as observed policy — no defect asserted without an authoritative rule</t>
         </is>
       </c>
-      <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2939,14 +3027,11 @@
           <t>Rejected or warned per configuration; actual behavior recorded</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr"/>
-      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3009,14 +3094,11 @@
           <t>Required-field message; no submission</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3079,14 +3161,11 @@
           <t>Status Cancelled; balance handling recorded as observed</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr"/>
-      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3149,14 +3228,11 @@
           <t>Status Approved in both views</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3219,14 +3295,11 @@
           <t>Status Rejected; comment visible to employee</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3289,14 +3362,11 @@
           <t>Actions unavailable or rejected with message</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3359,14 +3429,21 @@
           <t>Record with correct timestamp appears</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>ESS punch-in saves ("Successfully Saved") and creates visible attendance record with timestamp in My Records (1 row)</t>
+        </is>
+      </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>evidence/regression/REG-010-punched-in.png + REG-010-my-records.png</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3429,14 +3506,21 @@
           <t>End time + duration recorded and correct</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ESS punch-out saves ("Successfully Saved"), completing the in/out cycle the same day</t>
+        </is>
+      </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>evidence/regression/REG-010-punched-out.png</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3499,14 +3583,11 @@
           <t>Message shown; no orphan record created</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O44" t="inlineStr"/>
-      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3569,14 +3650,11 @@
           <t>Rejected or merged per observed rule; recorded</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3639,14 +3717,11 @@
           <t>Filter narrows correctly; data survives refresh</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O46" t="inlineStr"/>
-      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3709,14 +3784,11 @@
           <t>Vacancy listed with entered details</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O47" t="inlineStr"/>
-      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3779,14 +3851,11 @@
           <t>Inline errors; nothing created</t>
         </is>
       </c>
-      <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O48" t="inlineStr"/>
-      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3849,14 +3918,11 @@
           <t>Status updated; prior step retained in history</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3919,14 +3985,11 @@
           <t>Identical result sets and order</t>
         </is>
       </c>
-      <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O50" t="inlineStr"/>
-      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3989,14 +4052,11 @@
           <t>Rows match filters; counts sane</t>
         </is>
       </c>
-      <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4059,14 +4119,11 @@
           <t>Empty-state message; no error page or stale data</t>
         </is>
       </c>
-      <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O52" t="inlineStr"/>
-      <c r="P52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4129,14 +4186,11 @@
           <t>File downloads; row count matches screen</t>
         </is>
       </c>
-      <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4199,14 +4253,11 @@
           <t>Full path completable; focus visible throughout</t>
         </is>
       </c>
-      <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4269,14 +4320,11 @@
           <t>No branding/layout drift between modules or browsers</t>
         </is>
       </c>
-      <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>